<commit_message>
HPO 1024 points without exclusive rule
</commit_message>
<xml_diff>
--- a/dataset_agreed/saved_models/hyperparameter_optimized_runs/pointcloud_HPO_1024_run1/epoch_10/per_file_predictions_epoch_10.xlsx
+++ b/dataset_agreed/saved_models/hyperparameter_optimized_runs/pointcloud_HPO_1024_run1/epoch_10/per_file_predictions_epoch_10.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="520">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="521">
   <si>
     <t>Filename</t>
   </si>
@@ -808,772 +808,775 @@
     <t>0,1,1,0</t>
   </si>
   <si>
-    <t>0,1,0,1</t>
-  </si>
-  <si>
-    <t>0.7518,0.0426,0.0083,0.2484</t>
-  </si>
-  <si>
-    <t>0.0251,0.0110,0.0010,0.9852</t>
-  </si>
-  <si>
-    <t>0.8195,0.0762,0.0070,0.1266</t>
-  </si>
-  <si>
-    <t>0.1116,0.0058,0.0016,0.9479</t>
-  </si>
-  <si>
-    <t>0.9948,0.0056,0.0003,0.0006</t>
-  </si>
-  <si>
-    <t>0.9916,0.0070,0.0007,0.0014</t>
-  </si>
-  <si>
-    <t>0.9856,0.0121,0.0018,0.0017</t>
-  </si>
-  <si>
-    <t>0.9941,0.0035,0.0005,0.0016</t>
-  </si>
-  <si>
-    <t>0.9937,0.0058,0.0006,0.0008</t>
-  </si>
-  <si>
-    <t>0.9905,0.0098,0.0009,0.0010</t>
-  </si>
-  <si>
-    <t>0.9935,0.0064,0.0005,0.0007</t>
-  </si>
-  <si>
-    <t>0.9953,0.0041,0.0002,0.0008</t>
-  </si>
-  <si>
-    <t>0.7450,0.0731,0.1886,0.0607</t>
-  </si>
-  <si>
-    <t>0.2613,0.0728,0.7413,0.0388</t>
-  </si>
-  <si>
-    <t>0.2005,0.0808,0.8081,0.0166</t>
-  </si>
-  <si>
-    <t>0.1456,0.1203,0.7808,0.0131</t>
-  </si>
-  <si>
-    <t>0.6593,0.2351,0.1650,0.0380</t>
-  </si>
-  <si>
-    <t>0.1353,0.8875,0.0229,0.0033</t>
-  </si>
-  <si>
-    <t>0.2664,0.8050,0.0211,0.0058</t>
-  </si>
-  <si>
-    <t>0.7619,0.2481,0.0512,0.0065</t>
-  </si>
-  <si>
-    <t>0.1485,0.8869,0.0113,0.0056</t>
-  </si>
-  <si>
-    <t>0.0682,0.9488,0.0061,0.0022</t>
-  </si>
-  <si>
-    <t>0.4103,0.1330,0.4179,0.2128</t>
-  </si>
-  <si>
-    <t>0.2420,0.1286,0.5516,0.2547</t>
-  </si>
-  <si>
-    <t>0.0114,0.0195,0.9738,0.0129</t>
-  </si>
-  <si>
-    <t>0.1072,0.0208,0.7030,0.2099</t>
-  </si>
-  <si>
-    <t>0.0046,0.0140,0.9896,0.0050</t>
-  </si>
-  <si>
-    <t>0.2622,0.0220,0.4809,0.2182</t>
-  </si>
-  <si>
-    <t>0.0042,0.0098,0.9789,0.0323</t>
-  </si>
-  <si>
-    <t>0.4046,0.6875,0.0170,0.0033</t>
-  </si>
-  <si>
-    <t>0.5867,0.3798,0.0949,0.0164</t>
-  </si>
-  <si>
-    <t>0.0228,0.0467,0.9579,0.0198</t>
-  </si>
-  <si>
-    <t>0.0959,0.7781,0.1871,0.0080</t>
-  </si>
-  <si>
-    <t>0.8592,0.1445,0.0260,0.0093</t>
-  </si>
-  <si>
-    <t>0.1473,0.1384,0.7963,0.0215</t>
-  </si>
-  <si>
-    <t>0.6991,0.4354,0.0153,0.0042</t>
-  </si>
-  <si>
-    <t>0.2822,0.6554,0.1255,0.0116</t>
-  </si>
-  <si>
-    <t>0.0185,0.1452,0.9447,0.0214</t>
-  </si>
-  <si>
-    <t>0.0140,0.0420,0.8727,0.1672</t>
-  </si>
-  <si>
-    <t>0.0172,0.1424,0.7535,0.2432</t>
-  </si>
-  <si>
-    <t>0.0474,0.0241,0.8292,0.1855</t>
-  </si>
-  <si>
-    <t>0.0341,0.1150,0.9384,0.0075</t>
-  </si>
-  <si>
-    <t>0.0102,0.9586,0.0495,0.0132</t>
-  </si>
-  <si>
-    <t>0.0294,0.3119,0.8803,0.0184</t>
-  </si>
-  <si>
-    <t>0.1443,0.5230,0.0316,0.6105</t>
-  </si>
-  <si>
-    <t>0.0105,0.9720,0.0088,0.0296</t>
-  </si>
-  <si>
-    <t>0.0285,0.9433,0.0622,0.0255</t>
-  </si>
-  <si>
-    <t>0.0293,0.9477,0.0232,0.0521</t>
-  </si>
-  <si>
-    <t>0.0017,0.0066,0.9767,0.0500</t>
-  </si>
-  <si>
-    <t>0.0037,0.0474,0.9853,0.0071</t>
-  </si>
-  <si>
-    <t>0.0455,0.0825,0.9120,0.0353</t>
-  </si>
-  <si>
-    <t>0.1061,0.0341,0.8930,0.0161</t>
-  </si>
-  <si>
-    <t>0.0083,0.0155,0.9785,0.0144</t>
-  </si>
-  <si>
-    <t>0.0119,0.0251,0.9775,0.0106</t>
-  </si>
-  <si>
-    <t>0.9818,0.0241,0.0010,0.0021</t>
-  </si>
-  <si>
-    <t>0.9883,0.0103,0.0009,0.0020</t>
-  </si>
-  <si>
-    <t>0.9781,0.0200,0.0019,0.0037</t>
-  </si>
-  <si>
-    <t>0.0601,0.0728,0.9076,0.0335</t>
-  </si>
-  <si>
-    <t>0.9706,0.0286,0.0043,0.0028</t>
-  </si>
-  <si>
-    <t>0.9865,0.0108,0.0009,0.0033</t>
-  </si>
-  <si>
-    <t>0.9823,0.0186,0.0020,0.0016</t>
-  </si>
-  <si>
-    <t>0.0085,0.7765,0.8610,0.0061</t>
-  </si>
-  <si>
-    <t>0.0035,0.0217,0.9807,0.0190</t>
-  </si>
-  <si>
-    <t>0.0074,0.0806,0.9626,0.0236</t>
-  </si>
-  <si>
-    <t>0.0047,0.3632,0.9658,0.0069</t>
-  </si>
-  <si>
-    <t>0.0040,0.0121,0.9810,0.0226</t>
-  </si>
-  <si>
-    <t>0.0900,0.9099,0.0260,0.0074</t>
-  </si>
-  <si>
-    <t>0.0068,0.9880,0.0017,0.0025</t>
-  </si>
-  <si>
-    <t>0.4729,0.1879,0.4050,0.0144</t>
-  </si>
-  <si>
-    <t>0.6533,0.3152,0.1069,0.0385</t>
-  </si>
-  <si>
-    <t>0.0904,0.2270,0.7457,0.0207</t>
-  </si>
-  <si>
-    <t>0.0144,0.6826,0.8618,0.0101</t>
-  </si>
-  <si>
-    <t>0.0539,0.5966,0.7676,0.0361</t>
-  </si>
-  <si>
-    <t>0.0037,0.9767,0.1527,0.0061</t>
-  </si>
-  <si>
-    <t>0.0034,0.4677,0.9598,0.0035</t>
-  </si>
-  <si>
-    <t>0.0856,0.0082,0.0018,0.9579</t>
-  </si>
-  <si>
-    <t>0.0617,0.0032,0.0006,0.9754</t>
-  </si>
-  <si>
-    <t>0.0237,0.0128,0.0027,0.9837</t>
-  </si>
-  <si>
-    <t>0.0608,0.0064,0.0010,0.9716</t>
-  </si>
-  <si>
-    <t>0.0750,0.0047,0.0008,0.9690</t>
-  </si>
-  <si>
-    <t>0.0229,0.0052,0.0032,0.9826</t>
-  </si>
-  <si>
-    <t>0.0093,0.7952,0.8574,0.0095</t>
-  </si>
-  <si>
-    <t>0.0058,0.5484,0.9469,0.0057</t>
-  </si>
-  <si>
-    <t>0.0109,0.4296,0.9221,0.0073</t>
-  </si>
-  <si>
-    <t>0.0151,0.0790,0.9642,0.0129</t>
-  </si>
-  <si>
-    <t>0.0096,0.7683,0.8359,0.0055</t>
-  </si>
-  <si>
-    <t>0.0291,0.8513,0.4000,0.0511</t>
-  </si>
-  <si>
-    <t>0.9924,0.0067,0.0009,0.0009</t>
-  </si>
-  <si>
-    <t>0.9907,0.0101,0.0005,0.0012</t>
-  </si>
-  <si>
-    <t>0.9773,0.0240,0.0025,0.0020</t>
-  </si>
-  <si>
-    <t>0.9956,0.0034,0.0002,0.0008</t>
-  </si>
-  <si>
-    <t>0.9837,0.0084,0.0018,0.0057</t>
-  </si>
-  <si>
-    <t>0.9947,0.0048,0.0003,0.0009</t>
-  </si>
-  <si>
-    <t>0.9887,0.0085,0.0015,0.0017</t>
-  </si>
-  <si>
-    <t>0.9845,0.0170,0.0015,0.0017</t>
-  </si>
-  <si>
-    <t>0.9919,0.0062,0.0006,0.0017</t>
-  </si>
-  <si>
-    <t>0.9941,0.0046,0.0005,0.0010</t>
-  </si>
-  <si>
-    <t>0.9925,0.0058,0.0009,0.0011</t>
-  </si>
-  <si>
-    <t>0.9941,0.0035,0.0004,0.0016</t>
-  </si>
-  <si>
-    <t>0.9948,0.0043,0.0005,0.0008</t>
-  </si>
-  <si>
-    <t>0.9947,0.0041,0.0006,0.0008</t>
-  </si>
-  <si>
-    <t>0.9915,0.0062,0.0008,0.0018</t>
-  </si>
-  <si>
-    <t>0.9955,0.0043,0.0002,0.0007</t>
-  </si>
-  <si>
-    <t>0.0061,0.0236,0.9627,0.0511</t>
-  </si>
-  <si>
-    <t>0.2579,0.5570,0.2293,0.2174</t>
-  </si>
-  <si>
-    <t>0.3308,0.1118,0.6048,0.0570</t>
-  </si>
-  <si>
-    <t>0.0414,0.0372,0.8879,0.1130</t>
-  </si>
-  <si>
-    <t>0.2007,0.8502,0.0115,0.0026</t>
-  </si>
-  <si>
-    <t>0.1163,0.9278,0.0030,0.0023</t>
-  </si>
-  <si>
-    <t>0.2413,0.8338,0.0070,0.0030</t>
-  </si>
-  <si>
-    <t>0.4543,0.6337,0.0147,0.0334</t>
-  </si>
-  <si>
-    <t>0.2984,0.7548,0.0202,0.0066</t>
-  </si>
-  <si>
-    <t>0.1893,0.8648,0.0118,0.0037</t>
-  </si>
-  <si>
-    <t>0.9552,0.0447,0.0061,0.0065</t>
-  </si>
-  <si>
-    <t>0.7364,0.1054,0.1007,0.0942</t>
-  </si>
-  <si>
-    <t>0.0811,0.0438,0.8693,0.0599</t>
-  </si>
-  <si>
-    <t>0.2836,0.6583,0.0927,0.1131</t>
-  </si>
-  <si>
-    <t>0.5197,0.3147,0.1971,0.0404</t>
-  </si>
-  <si>
-    <t>0.4537,0.2199,0.0232,0.3999</t>
-  </si>
-  <si>
-    <t>0.0182,0.9703,0.0145,0.0123</t>
-  </si>
-  <si>
-    <t>0.0200,0.9263,0.0140,0.1218</t>
-  </si>
-  <si>
-    <t>0.1525,0.7871,0.0182,0.1238</t>
-  </si>
-  <si>
-    <t>0.0029,0.9906,0.0099,0.0092</t>
-  </si>
-  <si>
-    <t>0.2268,0.8189,0.0244,0.0051</t>
-  </si>
-  <si>
-    <t>0.8144,0.2503,0.0159,0.0027</t>
-  </si>
-  <si>
-    <t>0.4991,0.6492,0.0105,0.0026</t>
-  </si>
-  <si>
-    <t>0.9660,0.0337,0.0053,0.0043</t>
-  </si>
-  <si>
-    <t>0.9876,0.0096,0.0007,0.0034</t>
-  </si>
-  <si>
-    <t>0.9910,0.0093,0.0007,0.0012</t>
-  </si>
-  <si>
-    <t>0.9788,0.0201,0.0030,0.0025</t>
-  </si>
-  <si>
-    <t>0.9886,0.0090,0.0010,0.0023</t>
-  </si>
-  <si>
-    <t>0.9750,0.0183,0.0036,0.0057</t>
-  </si>
-  <si>
-    <t>0.9924,0.0049,0.0007,0.0019</t>
-  </si>
-  <si>
-    <t>0.9926,0.0041,0.0006,0.0022</t>
-  </si>
-  <si>
-    <t>0.0118,0.7617,0.7909,0.0120</t>
-  </si>
-  <si>
-    <t>0.0055,0.4556,0.9558,0.0040</t>
-  </si>
-  <si>
-    <t>0.0092,0.1156,0.9666,0.0111</t>
-  </si>
-  <si>
-    <t>0.0410,0.3989,0.8433,0.0292</t>
-  </si>
-  <si>
-    <t>0.6069,0.2191,0.2412,0.1112</t>
-  </si>
-  <si>
-    <t>0.5937,0.2315,0.2434,0.0419</t>
-  </si>
-  <si>
-    <t>0.4200,0.0304,0.6134,0.0560</t>
-  </si>
-  <si>
-    <t>0.3214,0.5563,0.1905,0.0906</t>
-  </si>
-  <si>
-    <t>0.0693,0.0087,0.0019,0.9625</t>
-  </si>
-  <si>
-    <t>0.0042,0.0021,0.0002,0.9978</t>
-  </si>
-  <si>
-    <t>0.0124,0.0075,0.0012,0.9918</t>
-  </si>
-  <si>
-    <t>0.0463,0.0054,0.0015,0.9754</t>
-  </si>
-  <si>
-    <t>0.0083,0.5721,0.9107,0.0146</t>
-  </si>
-  <si>
-    <t>0.9624,0.0502,0.0035,0.0028</t>
-  </si>
-  <si>
-    <t>0.8791,0.1780,0.0084,0.0045</t>
-  </si>
-  <si>
-    <t>0.9784,0.0169,0.0019,0.0053</t>
-  </si>
-  <si>
-    <t>0.9125,0.1576,0.0025,0.0043</t>
-  </si>
-  <si>
-    <t>0.9524,0.0382,0.0073,0.0084</t>
-  </si>
-  <si>
-    <t>0.7026,0.0515,0.0320,0.2713</t>
-  </si>
-  <si>
-    <t>0.9764,0.0163,0.0030,0.0055</t>
-  </si>
-  <si>
-    <t>0.0346,0.0673,0.9233,0.0333</t>
-  </si>
-  <si>
-    <t>0.7848,0.0058,0.0031,0.2692</t>
-  </si>
-  <si>
-    <t>0.7946,0.0459,0.0107,0.2008</t>
-  </si>
-  <si>
-    <t>0.1583,0.7648,0.0359,0.1543</t>
-  </si>
-  <si>
-    <t>0.8159,0.2061,0.0114,0.0280</t>
-  </si>
-  <si>
-    <t>0.7633,0.1964,0.0705,0.0244</t>
-  </si>
-  <si>
-    <t>0.3530,0.6847,0.0429,0.0209</t>
-  </si>
-  <si>
-    <t>0.4733,0.5704,0.0454,0.0158</t>
-  </si>
-  <si>
-    <t>0.5730,0.4480,0.0571,0.0164</t>
-  </si>
-  <si>
-    <t>0.9829,0.0179,0.0020,0.0017</t>
-  </si>
-  <si>
-    <t>0.9893,0.0083,0.0013,0.0017</t>
-  </si>
-  <si>
-    <t>0.9911,0.0062,0.0007,0.0021</t>
-  </si>
-  <si>
-    <t>0.9884,0.0079,0.0013,0.0027</t>
-  </si>
-  <si>
-    <t>0.9803,0.0177,0.0021,0.0029</t>
-  </si>
-  <si>
-    <t>0.9905,0.0109,0.0006,0.0010</t>
-  </si>
-  <si>
-    <t>0.9907,0.0054,0.0007,0.0029</t>
-  </si>
-  <si>
-    <t>0.9886,0.0060,0.0013,0.0031</t>
-  </si>
-  <si>
-    <t>0.3326,0.7485,0.0215,0.0040</t>
-  </si>
-  <si>
-    <t>0.9620,0.0455,0.0038,0.0027</t>
-  </si>
-  <si>
-    <t>0.9359,0.1007,0.0040,0.0021</t>
-  </si>
-  <si>
-    <t>0.2539,0.1387,0.6379,0.0044</t>
-  </si>
-  <si>
-    <t>0.9748,0.0271,0.0020,0.0036</t>
-  </si>
-  <si>
-    <t>0.9691,0.0296,0.0054,0.0027</t>
-  </si>
-  <si>
-    <t>0.9734,0.0326,0.0028,0.0016</t>
-  </si>
-  <si>
-    <t>0.9808,0.0164,0.0016,0.0029</t>
-  </si>
-  <si>
-    <t>0.0236,0.0197,0.9713,0.0077</t>
-  </si>
-  <si>
-    <t>0.9393,0.0721,0.0080,0.0034</t>
-  </si>
-  <si>
-    <t>0.0010,0.0052,0.9968,0.0024</t>
-  </si>
-  <si>
-    <t>0.0058,0.0385,0.9724,0.0207</t>
-  </si>
-  <si>
-    <t>0.0817,0.0503,0.9048,0.0230</t>
-  </si>
-  <si>
-    <t>0.0002,0.0117,0.9962,0.0046</t>
-  </si>
-  <si>
-    <t>0.0095,0.0107,0.9835,0.0085</t>
-  </si>
-  <si>
-    <t>0.0048,0.0094,0.9874,0.0086</t>
-  </si>
-  <si>
-    <t>0.0095,0.0609,0.9769,0.0055</t>
-  </si>
-  <si>
-    <t>0.4278,0.2193,0.4030,0.0127</t>
-  </si>
-  <si>
-    <t>0.0385,0.0791,0.9297,0.0096</t>
-  </si>
-  <si>
-    <t>0.4001,0.2802,0.3885,0.0434</t>
-  </si>
-  <si>
-    <t>0.0864,0.7926,0.2207,0.0061</t>
-  </si>
-  <si>
-    <t>0.2076,0.5619,0.2840,0.0163</t>
-  </si>
-  <si>
-    <t>0.2062,0.2517,0.5771,0.0516</t>
-  </si>
-  <si>
-    <t>0.5635,0.3298,0.1481,0.0783</t>
-  </si>
-  <si>
-    <t>0.4812,0.2338,0.3073,0.1458</t>
-  </si>
-  <si>
-    <t>0.8681,0.1957,0.0099,0.0048</t>
-  </si>
-  <si>
-    <t>0.7764,0.3336,0.0069,0.0022</t>
-  </si>
-  <si>
-    <t>0.9026,0.1526,0.0046,0.0049</t>
-  </si>
-  <si>
-    <t>0.9905,0.0082,0.0007,0.0022</t>
-  </si>
-  <si>
-    <t>0.9363,0.0913,0.0056,0.0026</t>
-  </si>
-  <si>
-    <t>0.5665,0.2073,0.2872,0.0618</t>
-  </si>
-  <si>
-    <t>0.6312,0.0557,0.3513,0.0600</t>
-  </si>
-  <si>
-    <t>0.2626,0.2048,0.1043,0.6523</t>
-  </si>
-  <si>
-    <t>0.4032,0.0533,0.4418,0.1721</t>
-  </si>
-  <si>
-    <t>0.4343,0.0686,0.1140,0.4639</t>
-  </si>
-  <si>
-    <t>0.1709,0.2548,0.6132,0.0985</t>
-  </si>
-  <si>
-    <t>0.0436,0.1374,0.8947,0.0513</t>
-  </si>
-  <si>
-    <t>0.0416,0.1086,0.9008,0.0638</t>
-  </si>
-  <si>
-    <t>0.0759,0.0415,0.7603,0.1815</t>
-  </si>
-  <si>
-    <t>0.0085,0.0634,0.9653,0.0259</t>
-  </si>
-  <si>
-    <t>0.9937,0.0046,0.0006,0.0013</t>
-  </si>
-  <si>
-    <t>0.9684,0.0299,0.0066,0.0021</t>
-  </si>
-  <si>
-    <t>0.9907,0.0077,0.0010,0.0014</t>
-  </si>
-  <si>
-    <t>0.9882,0.0126,0.0012,0.0011</t>
-  </si>
-  <si>
-    <t>0.9868,0.0141,0.0008,0.0020</t>
-  </si>
-  <si>
-    <t>0.9712,0.0280,0.0056,0.0026</t>
-  </si>
-  <si>
-    <t>0.9786,0.0188,0.0020,0.0043</t>
-  </si>
-  <si>
-    <t>0.9916,0.0081,0.0008,0.0011</t>
-  </si>
-  <si>
-    <t>0.2656,0.0577,0.7952,0.0109</t>
-  </si>
-  <si>
-    <t>0.8133,0.0860,0.1218,0.0108</t>
-  </si>
-  <si>
-    <t>0.9304,0.0473,0.0114,0.0136</t>
-  </si>
-  <si>
-    <t>0.0003,0.0038,0.9983,0.0015</t>
-  </si>
-  <si>
-    <t>0.0021,0.0121,0.9912,0.0087</t>
-  </si>
-  <si>
-    <t>0.0118,0.0324,0.9726,0.0135</t>
-  </si>
-  <si>
-    <t>0.0008,0.0112,0.9962,0.0024</t>
-  </si>
-  <si>
-    <t>0.1154,0.1425,0.7749,0.1235</t>
-  </si>
-  <si>
-    <t>0.0005,0.0035,0.9973,0.0042</t>
-  </si>
-  <si>
-    <t>0.0200,0.0615,0.9599,0.0126</t>
-  </si>
-  <si>
-    <t>0.3728,0.2925,0.3821,0.0426</t>
-  </si>
-  <si>
-    <t>0.4999,0.0979,0.4592,0.0854</t>
-  </si>
-  <si>
-    <t>0.3869,0.1316,0.5409,0.0699</t>
-  </si>
-  <si>
-    <t>0.6188,0.1487,0.2487,0.1049</t>
-  </si>
-  <si>
-    <t>0.9927,0.0069,0.0006,0.0011</t>
-  </si>
-  <si>
-    <t>0.9924,0.0077,0.0006,0.0010</t>
-  </si>
-  <si>
-    <t>0.9923,0.0072,0.0007,0.0010</t>
-  </si>
-  <si>
-    <t>0.9847,0.0150,0.0017,0.0017</t>
-  </si>
-  <si>
-    <t>0.9918,0.0048,0.0006,0.0026</t>
-  </si>
-  <si>
-    <t>0.9839,0.0146,0.0016,0.0022</t>
-  </si>
-  <si>
-    <t>0.9895,0.0093,0.0010,0.0018</t>
-  </si>
-  <si>
-    <t>0.9780,0.0217,0.0033,0.0023</t>
-  </si>
-  <si>
-    <t>0.0158,0.0991,0.9600,0.0074</t>
-  </si>
-  <si>
-    <t>0.0005,0.0043,0.9947,0.0096</t>
-  </si>
-  <si>
-    <t>0.0162,0.1941,0.9527,0.0082</t>
-  </si>
-  <si>
-    <t>0.1442,0.0525,0.8266,0.0529</t>
-  </si>
-  <si>
-    <t>0.0121,0.0338,0.9544,0.0526</t>
-  </si>
-  <si>
-    <t>0.0654,0.0516,0.8998,0.0533</t>
-  </si>
-  <si>
-    <t>0.2604,0.0580,0.5861,0.1668</t>
-  </si>
-  <si>
-    <t>0.0246,0.0624,0.9256,0.0549</t>
-  </si>
-  <si>
-    <t>0.4378,0.0218,0.0039,0.6939</t>
-  </si>
-  <si>
-    <t>0.0262,0.0368,0.0013,0.9816</t>
-  </si>
-  <si>
-    <t>0.1774,0.0078,0.0024,0.9017</t>
-  </si>
-  <si>
-    <t>0.0089,0.0011,0.0002,0.9958</t>
-  </si>
-  <si>
-    <t>0.0654,0.0067,0.0012,0.9673</t>
-  </si>
-  <si>
-    <t>0.4090,0.1084,0.0278,0.6027</t>
+    <t>0,0,0,0</t>
+  </si>
+  <si>
+    <t>1,1,0,0</t>
+  </si>
+  <si>
+    <t>0.7665,0.1213,0.0173,0.1534</t>
+  </si>
+  <si>
+    <t>0.0735,0.0100,0.0012,0.9647</t>
+  </si>
+  <si>
+    <t>0.4078,0.0181,0.0010,0.7555</t>
+  </si>
+  <si>
+    <t>0.2998,0.0147,0.0128,0.7561</t>
+  </si>
+  <si>
+    <t>0.9947,0.0050,0.0005,0.0006</t>
+  </si>
+  <si>
+    <t>0.9960,0.0038,0.0002,0.0007</t>
+  </si>
+  <si>
+    <t>0.9925,0.0044,0.0005,0.0021</t>
+  </si>
+  <si>
+    <t>0.9916,0.0072,0.0007,0.0014</t>
+  </si>
+  <si>
+    <t>0.9924,0.0068,0.0006,0.0011</t>
+  </si>
+  <si>
+    <t>0.9904,0.0083,0.0010,0.0014</t>
+  </si>
+  <si>
+    <t>0.9953,0.0042,0.0003,0.0008</t>
+  </si>
+  <si>
+    <t>0.9937,0.0054,0.0005,0.0011</t>
+  </si>
+  <si>
+    <t>0.7054,0.1114,0.2064,0.0622</t>
+  </si>
+  <si>
+    <t>0.0404,0.0697,0.9342,0.0133</t>
+  </si>
+  <si>
+    <t>0.4663,0.1951,0.3872,0.0193</t>
+  </si>
+  <si>
+    <t>0.3491,0.1089,0.6080,0.0509</t>
+  </si>
+  <si>
+    <t>0.7651,0.0799,0.1608,0.0592</t>
+  </si>
+  <si>
+    <t>0.0574,0.9552,0.0060,0.0018</t>
+  </si>
+  <si>
+    <t>0.2263,0.8340,0.0123,0.0065</t>
+  </si>
+  <si>
+    <t>0.8176,0.2502,0.0142,0.0047</t>
+  </si>
+  <si>
+    <t>0.2994,0.7946,0.0142,0.0023</t>
+  </si>
+  <si>
+    <t>0.1708,0.8825,0.0123,0.0034</t>
+  </si>
+  <si>
+    <t>0.1002,0.2423,0.1646,0.7814</t>
+  </si>
+  <si>
+    <t>0.3166,0.0774,0.6288,0.0812</t>
+  </si>
+  <si>
+    <t>0.0516,0.0075,0.9359,0.0284</t>
+  </si>
+  <si>
+    <t>0.0566,0.0143,0.8245,0.1568</t>
+  </si>
+  <si>
+    <t>0.0462,0.0363,0.9391,0.0142</t>
+  </si>
+  <si>
+    <t>0.1332,0.0240,0.8808,0.0286</t>
+  </si>
+  <si>
+    <t>0.0356,0.0928,0.9185,0.0254</t>
+  </si>
+  <si>
+    <t>0.1101,0.8824,0.0316,0.0090</t>
+  </si>
+  <si>
+    <t>0.3616,0.1468,0.5068,0.0051</t>
+  </si>
+  <si>
+    <t>0.0019,0.0249,0.9889,0.0080</t>
+  </si>
+  <si>
+    <t>0.1103,0.8723,0.0426,0.0112</t>
+  </si>
+  <si>
+    <t>0.8537,0.1055,0.0483,0.0244</t>
+  </si>
+  <si>
+    <t>0.0779,0.0961,0.9004,0.0325</t>
+  </si>
+  <si>
+    <t>0.8533,0.1782,0.0177,0.0045</t>
+  </si>
+  <si>
+    <t>0.2323,0.7508,0.0862,0.0073</t>
+  </si>
+  <si>
+    <t>0.0170,0.2854,0.9086,0.0406</t>
+  </si>
+  <si>
+    <t>0.0190,0.2994,0.9291,0.0197</t>
+  </si>
+  <si>
+    <t>0.0311,0.3601,0.6911,0.2108</t>
+  </si>
+  <si>
+    <t>0.0199,0.0639,0.9242,0.0664</t>
+  </si>
+  <si>
+    <t>0.0342,0.1585,0.9116,0.0296</t>
+  </si>
+  <si>
+    <t>0.0282,0.8895,0.1982,0.0317</t>
+  </si>
+  <si>
+    <t>0.1008,0.3091,0.7708,0.0330</t>
+  </si>
+  <si>
+    <t>0.2087,0.7038,0.0598,0.2258</t>
+  </si>
+  <si>
+    <t>0.0052,0.9844,0.0048,0.0169</t>
+  </si>
+  <si>
+    <t>0.0329,0.9462,0.0413,0.0138</t>
+  </si>
+  <si>
+    <t>0.0135,0.9506,0.0070,0.1049</t>
+  </si>
+  <si>
+    <t>0.0051,0.0333,0.9804,0.0129</t>
+  </si>
+  <si>
+    <t>0.0025,0.1206,0.9742,0.0172</t>
+  </si>
+  <si>
+    <t>0.1833,0.0617,0.8304,0.0193</t>
+  </si>
+  <si>
+    <t>0.0516,0.0411,0.9122,0.0393</t>
+  </si>
+  <si>
+    <t>0.0047,0.0125,0.9574,0.0752</t>
+  </si>
+  <si>
+    <t>0.0077,0.0287,0.9721,0.0197</t>
+  </si>
+  <si>
+    <t>0.9808,0.0192,0.0031,0.0023</t>
+  </si>
+  <si>
+    <t>0.9863,0.0128,0.0012,0.0024</t>
+  </si>
+  <si>
+    <t>0.9836,0.0186,0.0010,0.0021</t>
+  </si>
+  <si>
+    <t>0.0308,0.0266,0.9591,0.0145</t>
+  </si>
+  <si>
+    <t>0.9854,0.0129,0.0011,0.0031</t>
+  </si>
+  <si>
+    <t>0.9884,0.0142,0.0006,0.0013</t>
+  </si>
+  <si>
+    <t>0.9853,0.0151,0.0018,0.0012</t>
+  </si>
+  <si>
+    <t>0.0079,0.2627,0.9603,0.0137</t>
+  </si>
+  <si>
+    <t>0.0004,0.0096,0.9966,0.0027</t>
+  </si>
+  <si>
+    <t>0.0045,0.0230,0.9839,0.0117</t>
+  </si>
+  <si>
+    <t>0.0089,0.6865,0.8923,0.0066</t>
+  </si>
+  <si>
+    <t>0.0066,0.0105,0.9814,0.0185</t>
+  </si>
+  <si>
+    <t>0.0795,0.9245,0.0159,0.0075</t>
+  </si>
+  <si>
+    <t>0.0064,0.9893,0.0016,0.0014</t>
+  </si>
+  <si>
+    <t>0.9096,0.0610,0.0391,0.0132</t>
+  </si>
+  <si>
+    <t>0.3750,0.5999,0.0998,0.0249</t>
+  </si>
+  <si>
+    <t>0.1007,0.1685,0.7947,0.0120</t>
+  </si>
+  <si>
+    <t>0.0087,0.7643,0.8191,0.0094</t>
+  </si>
+  <si>
+    <t>0.0211,0.7326,0.8123,0.0118</t>
+  </si>
+  <si>
+    <t>0.0024,0.9762,0.1221,0.0194</t>
+  </si>
+  <si>
+    <t>0.0020,0.6810,0.9260,0.0059</t>
+  </si>
+  <si>
+    <t>0.0553,0.0042,0.0016,0.9708</t>
+  </si>
+  <si>
+    <t>0.1374,0.0048,0.0012,0.9364</t>
+  </si>
+  <si>
+    <t>0.0154,0.0068,0.0006,0.9919</t>
+  </si>
+  <si>
+    <t>0.0177,0.0055,0.0032,0.9862</t>
+  </si>
+  <si>
+    <t>0.1394,0.0173,0.0174,0.8916</t>
+  </si>
+  <si>
+    <t>0.0355,0.0075,0.0029,0.9775</t>
+  </si>
+  <si>
+    <t>0.0050,0.8627,0.7849,0.0088</t>
+  </si>
+  <si>
+    <t>0.0077,0.2313,0.9680,0.0077</t>
+  </si>
+  <si>
+    <t>0.0569,0.2060,0.8570,0.0570</t>
+  </si>
+  <si>
+    <t>0.0198,0.5184,0.9021,0.0083</t>
+  </si>
+  <si>
+    <t>0.0170,0.8993,0.5578,0.0087</t>
+  </si>
+  <si>
+    <t>0.0213,0.6785,0.7552,0.0317</t>
+  </si>
+  <si>
+    <t>0.9929,0.0063,0.0006,0.0011</t>
+  </si>
+  <si>
+    <t>0.9854,0.0185,0.0009,0.0014</t>
+  </si>
+  <si>
+    <t>0.9891,0.0085,0.0012,0.0020</t>
+  </si>
+  <si>
+    <t>0.9935,0.0062,0.0005,0.0010</t>
+  </si>
+  <si>
+    <t>0.9902,0.0074,0.0010,0.0019</t>
+  </si>
+  <si>
+    <t>0.9923,0.0069,0.0006,0.0013</t>
+  </si>
+  <si>
+    <t>0.9861,0.0149,0.0011,0.0019</t>
+  </si>
+  <si>
+    <t>0.9894,0.0108,0.0013,0.0010</t>
+  </si>
+  <si>
+    <t>0.9949,0.0038,0.0004,0.0009</t>
+  </si>
+  <si>
+    <t>0.9938,0.0051,0.0003,0.0016</t>
+  </si>
+  <si>
+    <t>0.9927,0.0066,0.0007,0.0009</t>
+  </si>
+  <si>
+    <t>0.9930,0.0071,0.0007,0.0006</t>
+  </si>
+  <si>
+    <t>0.9928,0.0059,0.0007,0.0013</t>
+  </si>
+  <si>
+    <t>0.9875,0.0120,0.0014,0.0011</t>
+  </si>
+  <si>
+    <t>0.9897,0.0078,0.0010,0.0023</t>
+  </si>
+  <si>
+    <t>0.9952,0.0039,0.0004,0.0009</t>
+  </si>
+  <si>
+    <t>0.0019,0.0048,0.9845,0.0313</t>
+  </si>
+  <si>
+    <t>0.0189,0.0357,0.8657,0.1799</t>
+  </si>
+  <si>
+    <t>0.5322,0.1428,0.1540,0.2682</t>
+  </si>
+  <si>
+    <t>0.0434,0.0567,0.9193,0.0393</t>
+  </si>
+  <si>
+    <t>0.3008,0.7847,0.0122,0.0034</t>
+  </si>
+  <si>
+    <t>0.2746,0.8055,0.0168,0.0037</t>
+  </si>
+  <si>
+    <t>0.6223,0.5305,0.0073,0.0022</t>
+  </si>
+  <si>
+    <t>0.8035,0.2931,0.0073,0.0025</t>
+  </si>
+  <si>
+    <t>0.0609,0.9407,0.0119,0.0032</t>
+  </si>
+  <si>
+    <t>0.0353,0.9647,0.0087,0.0026</t>
+  </si>
+  <si>
+    <t>0.8752,0.1974,0.0061,0.0025</t>
+  </si>
+  <si>
+    <t>0.6594,0.1994,0.1699,0.0169</t>
+  </si>
+  <si>
+    <t>0.3385,0.0308,0.6872,0.0527</t>
+  </si>
+  <si>
+    <t>0.5384,0.3044,0.1662,0.1398</t>
+  </si>
+  <si>
+    <t>0.5947,0.2578,0.1415,0.1260</t>
+  </si>
+  <si>
+    <t>0.2972,0.0625,0.0153,0.7593</t>
+  </si>
+  <si>
+    <t>0.0151,0.9778,0.0060,0.0069</t>
+  </si>
+  <si>
+    <t>0.0172,0.9625,0.0223,0.0320</t>
+  </si>
+  <si>
+    <t>0.3093,0.6829,0.0655,0.0782</t>
+  </si>
+  <si>
+    <t>0.0059,0.9765,0.0698,0.0213</t>
+  </si>
+  <si>
+    <t>0.1851,0.7841,0.1142,0.0070</t>
+  </si>
+  <si>
+    <t>0.8932,0.1310,0.0119,0.0028</t>
+  </si>
+  <si>
+    <t>0.5236,0.6014,0.0135,0.0031</t>
+  </si>
+  <si>
+    <t>0.9665,0.0228,0.0043,0.0078</t>
+  </si>
+  <si>
+    <t>0.9884,0.0099,0.0007,0.0027</t>
+  </si>
+  <si>
+    <t>0.9886,0.0071,0.0007,0.0039</t>
+  </si>
+  <si>
+    <t>0.9836,0.0143,0.0022,0.0024</t>
+  </si>
+  <si>
+    <t>0.9851,0.0128,0.0016,0.0022</t>
+  </si>
+  <si>
+    <t>0.9692,0.0263,0.0070,0.0035</t>
+  </si>
+  <si>
+    <t>0.9916,0.0070,0.0007,0.0013</t>
+  </si>
+  <si>
+    <t>0.9941,0.0042,0.0005,0.0015</t>
+  </si>
+  <si>
+    <t>0.0054,0.6944,0.9054,0.0051</t>
+  </si>
+  <si>
+    <t>0.0086,0.4221,0.9449,0.0053</t>
+  </si>
+  <si>
+    <t>0.0167,0.1721,0.9269,0.0364</t>
+  </si>
+  <si>
+    <t>0.0164,0.0663,0.9506,0.0300</t>
+  </si>
+  <si>
+    <t>0.4161,0.4524,0.1969,0.0719</t>
+  </si>
+  <si>
+    <t>0.5766,0.0731,0.4332,0.0485</t>
+  </si>
+  <si>
+    <t>0.5701,0.0190,0.3904,0.0725</t>
+  </si>
+  <si>
+    <t>0.5883,0.2879,0.1912,0.0836</t>
+  </si>
+  <si>
+    <t>0.1645,0.0135,0.0082,0.8834</t>
+  </si>
+  <si>
+    <t>0.0023,0.0015,0.0001,0.9987</t>
+  </si>
+  <si>
+    <t>0.0153,0.0129,0.0016,0.9890</t>
+  </si>
+  <si>
+    <t>0.0268,0.0041,0.0006,0.9879</t>
+  </si>
+  <si>
+    <t>0.0095,0.8383,0.6519,0.0236</t>
+  </si>
+  <si>
+    <t>0.9845,0.0115,0.0017,0.0029</t>
+  </si>
+  <si>
+    <t>0.8493,0.1973,0.0146,0.0073</t>
+  </si>
+  <si>
+    <t>0.9799,0.0283,0.0017,0.0010</t>
+  </si>
+  <si>
+    <t>0.9597,0.0430,0.0049,0.0043</t>
+  </si>
+  <si>
+    <t>0.9710,0.0213,0.0034,0.0059</t>
+  </si>
+  <si>
+    <t>0.7943,0.0101,0.0106,0.2025</t>
+  </si>
+  <si>
+    <t>0.9806,0.0107,0.0011,0.0080</t>
+  </si>
+  <si>
+    <t>0.0310,0.0442,0.8428,0.2142</t>
+  </si>
+  <si>
+    <t>0.7882,0.0122,0.0024,0.2968</t>
+  </si>
+  <si>
+    <t>0.8237,0.0345,0.0090,0.1642</t>
+  </si>
+  <si>
+    <t>0.1379,0.8118,0.0292,0.1150</t>
+  </si>
+  <si>
+    <t>0.8278,0.1205,0.0447,0.0306</t>
+  </si>
+  <si>
+    <t>0.6446,0.3508,0.0724,0.0158</t>
+  </si>
+  <si>
+    <t>0.5473,0.4318,0.0774,0.0156</t>
+  </si>
+  <si>
+    <t>0.7856,0.2020,0.0459,0.0108</t>
+  </si>
+  <si>
+    <t>0.6448,0.3834,0.0423,0.0600</t>
+  </si>
+  <si>
+    <t>0.9856,0.0108,0.0020,0.0019</t>
+  </si>
+  <si>
+    <t>0.9875,0.0109,0.0013,0.0020</t>
+  </si>
+  <si>
+    <t>0.9855,0.0095,0.0015,0.0037</t>
+  </si>
+  <si>
+    <t>0.9871,0.0094,0.0011,0.0039</t>
+  </si>
+  <si>
+    <t>0.9949,0.0040,0.0004,0.0009</t>
+  </si>
+  <si>
+    <t>0.9918,0.0064,0.0005,0.0020</t>
+  </si>
+  <si>
+    <t>0.9926,0.0045,0.0005,0.0024</t>
+  </si>
+  <si>
+    <t>0.9875,0.0109,0.0010,0.0023</t>
+  </si>
+  <si>
+    <t>0.6741,0.4458,0.0070,0.0057</t>
+  </si>
+  <si>
+    <t>0.8928,0.1385,0.0159,0.0051</t>
+  </si>
+  <si>
+    <t>0.9204,0.1213,0.0048,0.0030</t>
+  </si>
+  <si>
+    <t>0.8971,0.0895,0.0231,0.0051</t>
+  </si>
+  <si>
+    <t>0.9608,0.0402,0.0062,0.0031</t>
+  </si>
+  <si>
+    <t>0.9703,0.0303,0.0043,0.0028</t>
+  </si>
+  <si>
+    <t>0.9869,0.0113,0.0010,0.0025</t>
+  </si>
+  <si>
+    <t>0.9101,0.1350,0.0063,0.0024</t>
+  </si>
+  <si>
+    <t>0.0266,0.0441,0.9670,0.0029</t>
+  </si>
+  <si>
+    <t>0.9806,0.0235,0.0023,0.0015</t>
+  </si>
+  <si>
+    <t>0.0046,0.0084,0.9876,0.0109</t>
+  </si>
+  <si>
+    <t>0.0022,0.0179,0.9907,0.0061</t>
+  </si>
+  <si>
+    <t>0.0962,0.0234,0.8253,0.1213</t>
+  </si>
+  <si>
+    <t>0.0004,0.0211,0.9965,0.0022</t>
+  </si>
+  <si>
+    <t>0.0204,0.0729,0.9608,0.0046</t>
+  </si>
+  <si>
+    <t>0.0036,0.0100,0.9921,0.0040</t>
+  </si>
+  <si>
+    <t>0.0051,0.0031,0.9902,0.0079</t>
+  </si>
+  <si>
+    <t>0.5563,0.1393,0.2436,0.2220</t>
+  </si>
+  <si>
+    <t>0.2472,0.0849,0.7179,0.0450</t>
+  </si>
+  <si>
+    <t>0.5225,0.2330,0.2742,0.0692</t>
+  </si>
+  <si>
+    <t>0.1389,0.3246,0.5867,0.0060</t>
+  </si>
+  <si>
+    <t>0.1768,0.3064,0.5925,0.0108</t>
+  </si>
+  <si>
+    <t>0.5288,0.1366,0.3793,0.1445</t>
+  </si>
+  <si>
+    <t>0.2722,0.6155,0.1660,0.1315</t>
+  </si>
+  <si>
+    <t>0.4171,0.0910,0.5939,0.0451</t>
+  </si>
+  <si>
+    <t>0.9171,0.1352,0.0035,0.0023</t>
+  </si>
+  <si>
+    <t>0.7959,0.2664,0.0192,0.0058</t>
+  </si>
+  <si>
+    <t>0.9422,0.0798,0.0062,0.0022</t>
+  </si>
+  <si>
+    <t>0.9602,0.0433,0.0058,0.0036</t>
+  </si>
+  <si>
+    <t>0.9774,0.0318,0.0020,0.0019</t>
+  </si>
+  <si>
+    <t>0.6859,0.1234,0.2213,0.0677</t>
+  </si>
+  <si>
+    <t>0.3889,0.1027,0.1986,0.4347</t>
+  </si>
+  <si>
+    <t>0.6063,0.0687,0.2596,0.1257</t>
+  </si>
+  <si>
+    <t>0.4843,0.1405,0.4566,0.0664</t>
+  </si>
+  <si>
+    <t>0.1173,0.0379,0.8013,0.1417</t>
+  </si>
+  <si>
+    <t>0.0088,0.0647,0.9488,0.0405</t>
+  </si>
+  <si>
+    <t>0.0241,0.5624,0.4568,0.3519</t>
+  </si>
+  <si>
+    <t>0.0267,0.0730,0.9108,0.0804</t>
+  </si>
+  <si>
+    <t>0.0187,0.0906,0.9576,0.0190</t>
+  </si>
+  <si>
+    <t>0.0269,0.1698,0.8656,0.0813</t>
+  </si>
+  <si>
+    <t>0.9863,0.0093,0.0014,0.0034</t>
+  </si>
+  <si>
+    <t>0.9932,0.0061,0.0005,0.0008</t>
+  </si>
+  <si>
+    <t>0.9923,0.0075,0.0005,0.0012</t>
+  </si>
+  <si>
+    <t>0.9929,0.0068,0.0005,0.0011</t>
+  </si>
+  <si>
+    <t>0.9905,0.0083,0.0008,0.0017</t>
+  </si>
+  <si>
+    <t>0.9552,0.0744,0.0021,0.0016</t>
+  </si>
+  <si>
+    <t>0.9889,0.0078,0.0008,0.0027</t>
+  </si>
+  <si>
+    <t>0.9912,0.0080,0.0008,0.0015</t>
+  </si>
+  <si>
+    <t>0.4505,0.0447,0.6481,0.0180</t>
+  </si>
+  <si>
+    <t>0.4785,0.4602,0.0735,0.0049</t>
+  </si>
+  <si>
+    <t>0.8839,0.0374,0.0156,0.0722</t>
+  </si>
+  <si>
+    <t>0.0042,0.1287,0.9760,0.0042</t>
+  </si>
+  <si>
+    <t>0.0001,0.0030,0.9902,0.0381</t>
+  </si>
+  <si>
+    <t>0.0578,0.4871,0.6921,0.0196</t>
+  </si>
+  <si>
+    <t>0.0007,0.0036,0.9940,0.0111</t>
+  </si>
+  <si>
+    <t>0.0545,0.2404,0.8776,0.0170</t>
+  </si>
+  <si>
+    <t>0.0005,0.0036,0.9983,0.0014</t>
+  </si>
+  <si>
+    <t>0.0195,0.0505,0.9216,0.0674</t>
+  </si>
+  <si>
+    <t>0.1823,0.1247,0.7502,0.0244</t>
+  </si>
+  <si>
+    <t>0.6554,0.0246,0.1494,0.1378</t>
+  </si>
+  <si>
+    <t>0.2490,0.0502,0.2797,0.4778</t>
+  </si>
+  <si>
+    <t>0.3741,0.0278,0.0407,0.6031</t>
+  </si>
+  <si>
+    <t>0.9879,0.0093,0.0010,0.0025</t>
+  </si>
+  <si>
+    <t>0.9907,0.0086,0.0010,0.0016</t>
+  </si>
+  <si>
+    <t>0.9934,0.0054,0.0006,0.0008</t>
+  </si>
+  <si>
+    <t>0.9808,0.0193,0.0025,0.0018</t>
+  </si>
+  <si>
+    <t>0.9878,0.0123,0.0013,0.0017</t>
+  </si>
+  <si>
+    <t>0.9902,0.0090,0.0011,0.0010</t>
+  </si>
+  <si>
+    <t>0.9907,0.0069,0.0006,0.0027</t>
+  </si>
+  <si>
+    <t>0.9835,0.0185,0.0018,0.0015</t>
+  </si>
+  <si>
+    <t>0.0591,0.0838,0.9191,0.0245</t>
+  </si>
+  <si>
+    <t>0.0047,0.1345,0.9776,0.0036</t>
+  </si>
+  <si>
+    <t>0.0030,0.0323,0.9863,0.0084</t>
+  </si>
+  <si>
+    <t>0.1509,0.0449,0.8471,0.0234</t>
+  </si>
+  <si>
+    <t>0.0077,0.0090,0.9445,0.1050</t>
+  </si>
+  <si>
+    <t>0.2995,0.1583,0.4885,0.2367</t>
+  </si>
+  <si>
+    <t>0.1564,0.1098,0.6136,0.2818</t>
+  </si>
+  <si>
+    <t>0.0393,0.0460,0.3544,0.6884</t>
+  </si>
+  <si>
+    <t>0.6755,0.0112,0.0028,0.4365</t>
+  </si>
+  <si>
+    <t>0.0159,0.0084,0.0011,0.9898</t>
+  </si>
+  <si>
+    <t>0.1795,0.0138,0.0018,0.9149</t>
+  </si>
+  <si>
+    <t>0.0152,0.0050,0.0010,0.9909</t>
+  </si>
+  <si>
+    <t>0.0206,0.0017,0.0001,0.9925</t>
+  </si>
+  <si>
+    <t>0.4314,0.0101,0.0044,0.6748</t>
   </si>
 </sst>
 </file>
@@ -1959,7 +1962,7 @@
         <v>259</v>
       </c>
       <c r="D2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1973,7 +1976,7 @@
         <v>260</v>
       </c>
       <c r="D3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1984,10 +1987,10 @@
         <v>259</v>
       </c>
       <c r="C4" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D4" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -2001,7 +2004,7 @@
         <v>260</v>
       </c>
       <c r="D5" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -2015,7 +2018,7 @@
         <v>259</v>
       </c>
       <c r="D6" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -2029,7 +2032,7 @@
         <v>259</v>
       </c>
       <c r="D7" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -2043,7 +2046,7 @@
         <v>259</v>
       </c>
       <c r="D8" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -2057,7 +2060,7 @@
         <v>259</v>
       </c>
       <c r="D9" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -2071,7 +2074,7 @@
         <v>259</v>
       </c>
       <c r="D10" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -2085,7 +2088,7 @@
         <v>259</v>
       </c>
       <c r="D11" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -2099,7 +2102,7 @@
         <v>259</v>
       </c>
       <c r="D12" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -2113,7 +2116,7 @@
         <v>259</v>
       </c>
       <c r="D13" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -2127,7 +2130,7 @@
         <v>259</v>
       </c>
       <c r="D14" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -2141,7 +2144,7 @@
         <v>261</v>
       </c>
       <c r="D15" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -2152,10 +2155,10 @@
         <v>261</v>
       </c>
       <c r="C16" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="D16" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -2169,7 +2172,7 @@
         <v>261</v>
       </c>
       <c r="D17" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -2183,7 +2186,7 @@
         <v>259</v>
       </c>
       <c r="D18" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -2197,7 +2200,7 @@
         <v>262</v>
       </c>
       <c r="D19" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -2211,7 +2214,7 @@
         <v>262</v>
       </c>
       <c r="D20" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -2225,7 +2228,7 @@
         <v>259</v>
       </c>
       <c r="D21" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -2239,7 +2242,7 @@
         <v>262</v>
       </c>
       <c r="D22" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -2253,7 +2256,7 @@
         <v>262</v>
       </c>
       <c r="D23" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -2264,10 +2267,10 @@
         <v>259</v>
       </c>
       <c r="C24" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D24" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -2281,7 +2284,7 @@
         <v>261</v>
       </c>
       <c r="D25" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -2295,7 +2298,7 @@
         <v>261</v>
       </c>
       <c r="D26" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -2309,7 +2312,7 @@
         <v>261</v>
       </c>
       <c r="D27" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -2323,7 +2326,7 @@
         <v>261</v>
       </c>
       <c r="D28" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -2334,10 +2337,10 @@
         <v>261</v>
       </c>
       <c r="C29" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D29" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -2351,7 +2354,7 @@
         <v>261</v>
       </c>
       <c r="D30" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -2365,7 +2368,7 @@
         <v>262</v>
       </c>
       <c r="D31" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -2376,10 +2379,10 @@
         <v>259</v>
       </c>
       <c r="C32" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D32" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -2393,7 +2396,7 @@
         <v>261</v>
       </c>
       <c r="D33" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -2407,7 +2410,7 @@
         <v>262</v>
       </c>
       <c r="D34" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -2421,7 +2424,7 @@
         <v>259</v>
       </c>
       <c r="D35" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -2435,7 +2438,7 @@
         <v>261</v>
       </c>
       <c r="D36" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -2449,7 +2452,7 @@
         <v>259</v>
       </c>
       <c r="D37" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -2463,7 +2466,7 @@
         <v>262</v>
       </c>
       <c r="D38" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -2477,7 +2480,7 @@
         <v>261</v>
       </c>
       <c r="D39" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -2491,7 +2494,7 @@
         <v>261</v>
       </c>
       <c r="D40" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -2505,7 +2508,7 @@
         <v>261</v>
       </c>
       <c r="D41" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -2519,7 +2522,7 @@
         <v>261</v>
       </c>
       <c r="D42" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -2533,7 +2536,7 @@
         <v>261</v>
       </c>
       <c r="D43" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -2547,7 +2550,7 @@
         <v>262</v>
       </c>
       <c r="D44" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -2561,7 +2564,7 @@
         <v>261</v>
       </c>
       <c r="D45" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -2572,10 +2575,10 @@
         <v>259</v>
       </c>
       <c r="C46" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="D46" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -2589,7 +2592,7 @@
         <v>262</v>
       </c>
       <c r="D47" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -2603,7 +2606,7 @@
         <v>262</v>
       </c>
       <c r="D48" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -2617,7 +2620,7 @@
         <v>262</v>
       </c>
       <c r="D49" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -2631,7 +2634,7 @@
         <v>261</v>
       </c>
       <c r="D50" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -2645,7 +2648,7 @@
         <v>261</v>
       </c>
       <c r="D51" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -2659,7 +2662,7 @@
         <v>261</v>
       </c>
       <c r="D52" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -2673,7 +2676,7 @@
         <v>261</v>
       </c>
       <c r="D53" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="54" spans="1:4">
@@ -2687,7 +2690,7 @@
         <v>261</v>
       </c>
       <c r="D54" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="55" spans="1:4">
@@ -2701,7 +2704,7 @@
         <v>261</v>
       </c>
       <c r="D55" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -2715,7 +2718,7 @@
         <v>259</v>
       </c>
       <c r="D56" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -2729,7 +2732,7 @@
         <v>259</v>
       </c>
       <c r="D57" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="58" spans="1:4">
@@ -2743,7 +2746,7 @@
         <v>259</v>
       </c>
       <c r="D58" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="59" spans="1:4">
@@ -2757,7 +2760,7 @@
         <v>261</v>
       </c>
       <c r="D59" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="60" spans="1:4">
@@ -2771,7 +2774,7 @@
         <v>259</v>
       </c>
       <c r="D60" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="61" spans="1:4">
@@ -2785,7 +2788,7 @@
         <v>259</v>
       </c>
       <c r="D61" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="62" spans="1:4">
@@ -2799,7 +2802,7 @@
         <v>259</v>
       </c>
       <c r="D62" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="63" spans="1:4">
@@ -2810,10 +2813,10 @@
         <v>262</v>
       </c>
       <c r="C63" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D63" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="64" spans="1:4">
@@ -2827,7 +2830,7 @@
         <v>261</v>
       </c>
       <c r="D64" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="65" spans="1:4">
@@ -2841,7 +2844,7 @@
         <v>261</v>
       </c>
       <c r="D65" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="66" spans="1:4">
@@ -2852,10 +2855,10 @@
         <v>263</v>
       </c>
       <c r="C66" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D66" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="67" spans="1:4">
@@ -2869,7 +2872,7 @@
         <v>261</v>
       </c>
       <c r="D67" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="68" spans="1:4">
@@ -2883,7 +2886,7 @@
         <v>262</v>
       </c>
       <c r="D68" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="69" spans="1:4">
@@ -2897,7 +2900,7 @@
         <v>262</v>
       </c>
       <c r="D69" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="70" spans="1:4">
@@ -2911,7 +2914,7 @@
         <v>259</v>
       </c>
       <c r="D70" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="71" spans="1:4">
@@ -2922,10 +2925,10 @@
         <v>261</v>
       </c>
       <c r="C71" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D71" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="72" spans="1:4">
@@ -2939,7 +2942,7 @@
         <v>261</v>
       </c>
       <c r="D72" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="73" spans="1:4">
@@ -2953,7 +2956,7 @@
         <v>263</v>
       </c>
       <c r="D73" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="74" spans="1:4">
@@ -2967,7 +2970,7 @@
         <v>263</v>
       </c>
       <c r="D74" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="75" spans="1:4">
@@ -2981,7 +2984,7 @@
         <v>262</v>
       </c>
       <c r="D75" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="76" spans="1:4">
@@ -2992,10 +2995,10 @@
         <v>262</v>
       </c>
       <c r="C76" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D76" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="77" spans="1:4">
@@ -3009,7 +3012,7 @@
         <v>260</v>
       </c>
       <c r="D77" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="78" spans="1:4">
@@ -3023,7 +3026,7 @@
         <v>260</v>
       </c>
       <c r="D78" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="79" spans="1:4">
@@ -3037,7 +3040,7 @@
         <v>260</v>
       </c>
       <c r="D79" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="80" spans="1:4">
@@ -3051,7 +3054,7 @@
         <v>260</v>
       </c>
       <c r="D80" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
     </row>
     <row r="81" spans="1:4">
@@ -3065,7 +3068,7 @@
         <v>260</v>
       </c>
       <c r="D81" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="82" spans="1:4">
@@ -3079,7 +3082,7 @@
         <v>260</v>
       </c>
       <c r="D82" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="83" spans="1:4">
@@ -3093,7 +3096,7 @@
         <v>263</v>
       </c>
       <c r="D83" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="84" spans="1:4">
@@ -3104,10 +3107,10 @@
         <v>261</v>
       </c>
       <c r="C84" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D84" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="85" spans="1:4">
@@ -3121,7 +3124,7 @@
         <v>261</v>
       </c>
       <c r="D85" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="86" spans="1:4">
@@ -3132,10 +3135,10 @@
         <v>263</v>
       </c>
       <c r="C86" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D86" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="87" spans="1:4">
@@ -3149,7 +3152,7 @@
         <v>263</v>
       </c>
       <c r="D87" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="88" spans="1:4">
@@ -3160,10 +3163,10 @@
         <v>262</v>
       </c>
       <c r="C88" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D88" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="89" spans="1:4">
@@ -3177,7 +3180,7 @@
         <v>259</v>
       </c>
       <c r="D89" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
     </row>
     <row r="90" spans="1:4">
@@ -3191,7 +3194,7 @@
         <v>259</v>
       </c>
       <c r="D90" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="91" spans="1:4">
@@ -3205,7 +3208,7 @@
         <v>259</v>
       </c>
       <c r="D91" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="92" spans="1:4">
@@ -3219,7 +3222,7 @@
         <v>259</v>
       </c>
       <c r="D92" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="93" spans="1:4">
@@ -3233,7 +3236,7 @@
         <v>259</v>
       </c>
       <c r="D93" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="94" spans="1:4">
@@ -3247,7 +3250,7 @@
         <v>259</v>
       </c>
       <c r="D94" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="95" spans="1:4">
@@ -3261,7 +3264,7 @@
         <v>259</v>
       </c>
       <c r="D95" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="96" spans="1:4">
@@ -3275,7 +3278,7 @@
         <v>259</v>
       </c>
       <c r="D96" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="97" spans="1:4">
@@ -3289,7 +3292,7 @@
         <v>259</v>
       </c>
       <c r="D97" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="98" spans="1:4">
@@ -3303,7 +3306,7 @@
         <v>259</v>
       </c>
       <c r="D98" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="99" spans="1:4">
@@ -3317,7 +3320,7 @@
         <v>259</v>
       </c>
       <c r="D99" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="100" spans="1:4">
@@ -3331,7 +3334,7 @@
         <v>259</v>
       </c>
       <c r="D100" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="101" spans="1:4">
@@ -3345,7 +3348,7 @@
         <v>259</v>
       </c>
       <c r="D101" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="102" spans="1:4">
@@ -3359,7 +3362,7 @@
         <v>259</v>
       </c>
       <c r="D102" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="103" spans="1:4">
@@ -3373,7 +3376,7 @@
         <v>259</v>
       </c>
       <c r="D103" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="104" spans="1:4">
@@ -3387,7 +3390,7 @@
         <v>259</v>
       </c>
       <c r="D104" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="105" spans="1:4">
@@ -3401,7 +3404,7 @@
         <v>261</v>
       </c>
       <c r="D105" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="106" spans="1:4">
@@ -3412,10 +3415,10 @@
         <v>261</v>
       </c>
       <c r="C106" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D106" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="107" spans="1:4">
@@ -3426,10 +3429,10 @@
         <v>259</v>
       </c>
       <c r="C107" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D107" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="108" spans="1:4">
@@ -3443,7 +3446,7 @@
         <v>261</v>
       </c>
       <c r="D108" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="109" spans="1:4">
@@ -3457,7 +3460,7 @@
         <v>262</v>
       </c>
       <c r="D109" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="110" spans="1:4">
@@ -3471,7 +3474,7 @@
         <v>262</v>
       </c>
       <c r="D110" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
     </row>
     <row r="111" spans="1:4">
@@ -3482,10 +3485,10 @@
         <v>262</v>
       </c>
       <c r="C111" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="D111" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
     </row>
     <row r="112" spans="1:4">
@@ -3496,10 +3499,10 @@
         <v>262</v>
       </c>
       <c r="C112" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D112" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
     </row>
     <row r="113" spans="1:4">
@@ -3513,7 +3516,7 @@
         <v>262</v>
       </c>
       <c r="D113" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="114" spans="1:4">
@@ -3527,7 +3530,7 @@
         <v>262</v>
       </c>
       <c r="D114" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
     </row>
     <row r="115" spans="1:4">
@@ -3541,7 +3544,7 @@
         <v>259</v>
       </c>
       <c r="D115" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="116" spans="1:4">
@@ -3555,7 +3558,7 @@
         <v>259</v>
       </c>
       <c r="D116" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
     </row>
     <row r="117" spans="1:4">
@@ -3569,7 +3572,7 @@
         <v>261</v>
       </c>
       <c r="D117" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="118" spans="1:4">
@@ -3580,10 +3583,10 @@
         <v>259</v>
       </c>
       <c r="C118" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D118" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="119" spans="1:4">
@@ -3597,7 +3600,7 @@
         <v>259</v>
       </c>
       <c r="D119" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="120" spans="1:4">
@@ -3608,10 +3611,10 @@
         <v>262</v>
       </c>
       <c r="C120" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D120" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="121" spans="1:4">
@@ -3625,7 +3628,7 @@
         <v>262</v>
       </c>
       <c r="D121" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
     </row>
     <row r="122" spans="1:4">
@@ -3639,7 +3642,7 @@
         <v>262</v>
       </c>
       <c r="D122" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="123" spans="1:4">
@@ -3653,7 +3656,7 @@
         <v>262</v>
       </c>
       <c r="D123" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="124" spans="1:4">
@@ -3667,7 +3670,7 @@
         <v>262</v>
       </c>
       <c r="D124" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
     </row>
     <row r="125" spans="1:4">
@@ -3681,7 +3684,7 @@
         <v>262</v>
       </c>
       <c r="D125" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="126" spans="1:4">
@@ -3695,7 +3698,7 @@
         <v>259</v>
       </c>
       <c r="D126" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
     </row>
     <row r="127" spans="1:4">
@@ -3706,10 +3709,10 @@
         <v>259</v>
       </c>
       <c r="C127" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="D127" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="128" spans="1:4">
@@ -3723,7 +3726,7 @@
         <v>259</v>
       </c>
       <c r="D128" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="129" spans="1:4">
@@ -3737,7 +3740,7 @@
         <v>259</v>
       </c>
       <c r="D129" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
     </row>
     <row r="130" spans="1:4">
@@ -3751,7 +3754,7 @@
         <v>259</v>
       </c>
       <c r="D130" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="131" spans="1:4">
@@ -3765,7 +3768,7 @@
         <v>259</v>
       </c>
       <c r="D131" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
     </row>
     <row r="132" spans="1:4">
@@ -3779,7 +3782,7 @@
         <v>259</v>
       </c>
       <c r="D132" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
     </row>
     <row r="133" spans="1:4">
@@ -3793,7 +3796,7 @@
         <v>259</v>
       </c>
       <c r="D133" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="134" spans="1:4">
@@ -3807,7 +3810,7 @@
         <v>259</v>
       </c>
       <c r="D134" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
     </row>
     <row r="135" spans="1:4">
@@ -3821,7 +3824,7 @@
         <v>259</v>
       </c>
       <c r="D135" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="136" spans="1:4">
@@ -3835,7 +3838,7 @@
         <v>263</v>
       </c>
       <c r="D136" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
     </row>
     <row r="137" spans="1:4">
@@ -3849,7 +3852,7 @@
         <v>261</v>
       </c>
       <c r="D137" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="138" spans="1:4">
@@ -3863,7 +3866,7 @@
         <v>261</v>
       </c>
       <c r="D138" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="139" spans="1:4">
@@ -3877,7 +3880,7 @@
         <v>261</v>
       </c>
       <c r="D139" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="140" spans="1:4">
@@ -3888,10 +3891,10 @@
         <v>259</v>
       </c>
       <c r="C140" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D140" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
     </row>
     <row r="141" spans="1:4">
@@ -3905,7 +3908,7 @@
         <v>259</v>
       </c>
       <c r="D141" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="142" spans="1:4">
@@ -3916,10 +3919,10 @@
         <v>261</v>
       </c>
       <c r="C142" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D142" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
     <row r="143" spans="1:4">
@@ -3930,10 +3933,10 @@
         <v>259</v>
       </c>
       <c r="C143" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D143" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="144" spans="1:4">
@@ -3947,7 +3950,7 @@
         <v>260</v>
       </c>
       <c r="D144" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
     <row r="145" spans="1:4">
@@ -3961,7 +3964,7 @@
         <v>260</v>
       </c>
       <c r="D145" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
     </row>
     <row r="146" spans="1:4">
@@ -3975,7 +3978,7 @@
         <v>260</v>
       </c>
       <c r="D146" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="147" spans="1:4">
@@ -3989,7 +3992,7 @@
         <v>260</v>
       </c>
       <c r="D147" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="148" spans="1:4">
@@ -4003,7 +4006,7 @@
         <v>263</v>
       </c>
       <c r="D148" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="149" spans="1:4">
@@ -4017,7 +4020,7 @@
         <v>259</v>
       </c>
       <c r="D149" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
     </row>
     <row r="150" spans="1:4">
@@ -4031,7 +4034,7 @@
         <v>259</v>
       </c>
       <c r="D150" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
     </row>
     <row r="151" spans="1:4">
@@ -4045,7 +4048,7 @@
         <v>259</v>
       </c>
       <c r="D151" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
     </row>
     <row r="152" spans="1:4">
@@ -4059,7 +4062,7 @@
         <v>259</v>
       </c>
       <c r="D152" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
     </row>
     <row r="153" spans="1:4">
@@ -4073,7 +4076,7 @@
         <v>259</v>
       </c>
       <c r="D153" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
     </row>
     <row r="154" spans="1:4">
@@ -4087,7 +4090,7 @@
         <v>259</v>
       </c>
       <c r="D154" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
     </row>
     <row r="155" spans="1:4">
@@ -4101,7 +4104,7 @@
         <v>259</v>
       </c>
       <c r="D155" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
     </row>
     <row r="156" spans="1:4">
@@ -4115,7 +4118,7 @@
         <v>261</v>
       </c>
       <c r="D156" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
     </row>
     <row r="157" spans="1:4">
@@ -4129,7 +4132,7 @@
         <v>259</v>
       </c>
       <c r="D157" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
     </row>
     <row r="158" spans="1:4">
@@ -4143,7 +4146,7 @@
         <v>259</v>
       </c>
       <c r="D158" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="159" spans="1:4">
@@ -4157,7 +4160,7 @@
         <v>262</v>
       </c>
       <c r="D159" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
     </row>
     <row r="160" spans="1:4">
@@ -4171,7 +4174,7 @@
         <v>259</v>
       </c>
       <c r="D160" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
     </row>
     <row r="161" spans="1:4">
@@ -4185,7 +4188,7 @@
         <v>259</v>
       </c>
       <c r="D161" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
     <row r="162" spans="1:4">
@@ -4196,10 +4199,10 @@
         <v>262</v>
       </c>
       <c r="C162" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D162" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
     </row>
     <row r="163" spans="1:4">
@@ -4210,10 +4213,10 @@
         <v>259</v>
       </c>
       <c r="C163" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D163" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
     </row>
     <row r="164" spans="1:4">
@@ -4227,7 +4230,7 @@
         <v>259</v>
       </c>
       <c r="D164" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
     </row>
     <row r="165" spans="1:4">
@@ -4241,7 +4244,7 @@
         <v>259</v>
       </c>
       <c r="D165" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
     </row>
     <row r="166" spans="1:4">
@@ -4255,7 +4258,7 @@
         <v>259</v>
       </c>
       <c r="D166" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="167" spans="1:4">
@@ -4269,7 +4272,7 @@
         <v>259</v>
       </c>
       <c r="D167" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
     </row>
     <row r="168" spans="1:4">
@@ -4283,7 +4286,7 @@
         <v>259</v>
       </c>
       <c r="D168" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="169" spans="1:4">
@@ -4297,7 +4300,7 @@
         <v>259</v>
       </c>
       <c r="D169" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
     </row>
     <row r="170" spans="1:4">
@@ -4311,7 +4314,7 @@
         <v>259</v>
       </c>
       <c r="D170" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
     </row>
     <row r="171" spans="1:4">
@@ -4325,7 +4328,7 @@
         <v>259</v>
       </c>
       <c r="D171" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
     </row>
     <row r="172" spans="1:4">
@@ -4339,7 +4342,7 @@
         <v>259</v>
       </c>
       <c r="D172" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
     </row>
     <row r="173" spans="1:4">
@@ -4350,10 +4353,10 @@
         <v>259</v>
       </c>
       <c r="C173" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D173" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="174" spans="1:4">
@@ -4367,7 +4370,7 @@
         <v>259</v>
       </c>
       <c r="D174" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="175" spans="1:4">
@@ -4381,7 +4384,7 @@
         <v>259</v>
       </c>
       <c r="D175" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
     </row>
     <row r="176" spans="1:4">
@@ -4392,10 +4395,10 @@
         <v>261</v>
       </c>
       <c r="C176" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D176" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="177" spans="1:4">
@@ -4409,7 +4412,7 @@
         <v>259</v>
       </c>
       <c r="D177" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="178" spans="1:4">
@@ -4423,7 +4426,7 @@
         <v>259</v>
       </c>
       <c r="D178" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="179" spans="1:4">
@@ -4437,7 +4440,7 @@
         <v>259</v>
       </c>
       <c r="D179" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
     </row>
     <row r="180" spans="1:4">
@@ -4451,7 +4454,7 @@
         <v>259</v>
       </c>
       <c r="D180" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
     </row>
     <row r="181" spans="1:4">
@@ -4465,7 +4468,7 @@
         <v>261</v>
       </c>
       <c r="D181" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
     </row>
     <row r="182" spans="1:4">
@@ -4479,7 +4482,7 @@
         <v>259</v>
       </c>
       <c r="D182" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
     </row>
     <row r="183" spans="1:4">
@@ -4493,7 +4496,7 @@
         <v>261</v>
       </c>
       <c r="D183" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
     </row>
     <row r="184" spans="1:4">
@@ -4507,7 +4510,7 @@
         <v>261</v>
       </c>
       <c r="D184" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="185" spans="1:4">
@@ -4521,7 +4524,7 @@
         <v>261</v>
       </c>
       <c r="D185" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
     </row>
     <row r="186" spans="1:4">
@@ -4535,7 +4538,7 @@
         <v>261</v>
       </c>
       <c r="D186" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="187" spans="1:4">
@@ -4549,7 +4552,7 @@
         <v>261</v>
       </c>
       <c r="D187" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
     </row>
     <row r="188" spans="1:4">
@@ -4563,7 +4566,7 @@
         <v>261</v>
       </c>
       <c r="D188" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="189" spans="1:4">
@@ -4577,7 +4580,7 @@
         <v>261</v>
       </c>
       <c r="D189" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
     </row>
     <row r="190" spans="1:4">
@@ -4591,7 +4594,7 @@
         <v>259</v>
       </c>
       <c r="D190" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
     </row>
     <row r="191" spans="1:4">
@@ -4605,7 +4608,7 @@
         <v>261</v>
       </c>
       <c r="D191" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
     </row>
     <row r="192" spans="1:4">
@@ -4619,7 +4622,7 @@
         <v>259</v>
       </c>
       <c r="D192" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
     </row>
     <row r="193" spans="1:4">
@@ -4630,10 +4633,10 @@
         <v>261</v>
       </c>
       <c r="C193" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D193" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
     </row>
     <row r="194" spans="1:4">
@@ -4644,10 +4647,10 @@
         <v>261</v>
       </c>
       <c r="C194" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D194" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
     </row>
     <row r="195" spans="1:4">
@@ -4658,10 +4661,10 @@
         <v>261</v>
       </c>
       <c r="C195" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D195" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
     </row>
     <row r="196" spans="1:4">
@@ -4672,10 +4675,10 @@
         <v>259</v>
       </c>
       <c r="C196" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D196" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
     </row>
     <row r="197" spans="1:4">
@@ -4686,10 +4689,10 @@
         <v>259</v>
       </c>
       <c r="C197" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D197" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
     </row>
     <row r="198" spans="1:4">
@@ -4703,7 +4706,7 @@
         <v>259</v>
       </c>
       <c r="D198" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
     </row>
     <row r="199" spans="1:4">
@@ -4717,7 +4720,7 @@
         <v>259</v>
       </c>
       <c r="D199" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
     </row>
     <row r="200" spans="1:4">
@@ -4731,7 +4734,7 @@
         <v>259</v>
       </c>
       <c r="D200" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
     </row>
     <row r="201" spans="1:4">
@@ -4745,7 +4748,7 @@
         <v>259</v>
       </c>
       <c r="D201" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
     </row>
     <row r="202" spans="1:4">
@@ -4759,7 +4762,7 @@
         <v>259</v>
       </c>
       <c r="D202" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
     </row>
     <row r="203" spans="1:4">
@@ -4773,7 +4776,7 @@
         <v>259</v>
       </c>
       <c r="D203" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
     </row>
     <row r="204" spans="1:4">
@@ -4784,10 +4787,10 @@
         <v>259</v>
       </c>
       <c r="C204" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D204" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
     </row>
     <row r="205" spans="1:4">
@@ -4798,10 +4801,10 @@
         <v>259</v>
       </c>
       <c r="C205" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D205" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="206" spans="1:4">
@@ -4812,10 +4815,10 @@
         <v>261</v>
       </c>
       <c r="C206" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D206" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
     </row>
     <row r="207" spans="1:4">
@@ -4826,10 +4829,10 @@
         <v>259</v>
       </c>
       <c r="C207" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D207" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
     </row>
     <row r="208" spans="1:4">
@@ -4843,7 +4846,7 @@
         <v>261</v>
       </c>
       <c r="D208" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
     </row>
     <row r="209" spans="1:4">
@@ -4854,10 +4857,10 @@
         <v>261</v>
       </c>
       <c r="C209" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D209" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
     </row>
     <row r="210" spans="1:4">
@@ -4871,7 +4874,7 @@
         <v>261</v>
       </c>
       <c r="D210" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="211" spans="1:4">
@@ -4885,7 +4888,7 @@
         <v>261</v>
       </c>
       <c r="D211" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="212" spans="1:4">
@@ -4899,7 +4902,7 @@
         <v>261</v>
       </c>
       <c r="D212" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
     </row>
     <row r="213" spans="1:4">
@@ -4913,7 +4916,7 @@
         <v>259</v>
       </c>
       <c r="D213" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
     </row>
     <row r="214" spans="1:4">
@@ -4927,7 +4930,7 @@
         <v>259</v>
       </c>
       <c r="D214" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
     </row>
     <row r="215" spans="1:4">
@@ -4941,7 +4944,7 @@
         <v>259</v>
       </c>
       <c r="D215" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
     </row>
     <row r="216" spans="1:4">
@@ -4955,7 +4958,7 @@
         <v>259</v>
       </c>
       <c r="D216" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
     </row>
     <row r="217" spans="1:4">
@@ -4969,7 +4972,7 @@
         <v>259</v>
       </c>
       <c r="D217" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
     </row>
     <row r="218" spans="1:4">
@@ -4983,7 +4986,7 @@
         <v>259</v>
       </c>
       <c r="D218" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
     </row>
     <row r="219" spans="1:4">
@@ -4997,7 +5000,7 @@
         <v>259</v>
       </c>
       <c r="D219" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
     </row>
     <row r="220" spans="1:4">
@@ -5011,7 +5014,7 @@
         <v>259</v>
       </c>
       <c r="D220" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
     </row>
     <row r="221" spans="1:4">
@@ -5025,7 +5028,7 @@
         <v>261</v>
       </c>
       <c r="D221" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
     </row>
     <row r="222" spans="1:4">
@@ -5036,10 +5039,10 @@
         <v>259</v>
       </c>
       <c r="C222" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D222" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
     </row>
     <row r="223" spans="1:4">
@@ -5053,7 +5056,7 @@
         <v>259</v>
       </c>
       <c r="D223" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
     </row>
     <row r="224" spans="1:4">
@@ -5067,7 +5070,7 @@
         <v>261</v>
       </c>
       <c r="D224" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
     </row>
     <row r="225" spans="1:4">
@@ -5081,7 +5084,7 @@
         <v>261</v>
       </c>
       <c r="D225" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
     <row r="226" spans="1:4">
@@ -5095,7 +5098,7 @@
         <v>261</v>
       </c>
       <c r="D226" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
     </row>
     <row r="227" spans="1:4">
@@ -5109,7 +5112,7 @@
         <v>261</v>
       </c>
       <c r="D227" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
     </row>
     <row r="228" spans="1:4">
@@ -5123,7 +5126,7 @@
         <v>261</v>
       </c>
       <c r="D228" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
     </row>
     <row r="229" spans="1:4">
@@ -5137,7 +5140,7 @@
         <v>261</v>
       </c>
       <c r="D229" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
     </row>
     <row r="230" spans="1:4">
@@ -5151,7 +5154,7 @@
         <v>261</v>
       </c>
       <c r="D230" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
     </row>
     <row r="231" spans="1:4">
@@ -5162,10 +5165,10 @@
         <v>261</v>
       </c>
       <c r="C231" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D231" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
     </row>
     <row r="232" spans="1:4">
@@ -5179,7 +5182,7 @@
         <v>259</v>
       </c>
       <c r="D232" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
     </row>
     <row r="233" spans="1:4">
@@ -5190,10 +5193,10 @@
         <v>259</v>
       </c>
       <c r="C233" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="D233" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
     </row>
     <row r="234" spans="1:4">
@@ -5204,10 +5207,10 @@
         <v>259</v>
       </c>
       <c r="C234" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D234" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
     </row>
     <row r="235" spans="1:4">
@@ -5221,7 +5224,7 @@
         <v>259</v>
       </c>
       <c r="D235" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
     </row>
     <row r="236" spans="1:4">
@@ -5235,7 +5238,7 @@
         <v>259</v>
       </c>
       <c r="D236" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
     </row>
     <row r="237" spans="1:4">
@@ -5249,7 +5252,7 @@
         <v>259</v>
       </c>
       <c r="D237" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
     </row>
     <row r="238" spans="1:4">
@@ -5263,7 +5266,7 @@
         <v>259</v>
       </c>
       <c r="D238" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
     </row>
     <row r="239" spans="1:4">
@@ -5277,7 +5280,7 @@
         <v>259</v>
       </c>
       <c r="D239" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
     </row>
     <row r="240" spans="1:4">
@@ -5291,7 +5294,7 @@
         <v>259</v>
       </c>
       <c r="D240" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
     </row>
     <row r="241" spans="1:4">
@@ -5305,7 +5308,7 @@
         <v>259</v>
       </c>
       <c r="D241" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
     </row>
     <row r="242" spans="1:4">
@@ -5319,7 +5322,7 @@
         <v>259</v>
       </c>
       <c r="D242" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
     </row>
     <row r="243" spans="1:4">
@@ -5333,7 +5336,7 @@
         <v>261</v>
       </c>
       <c r="D243" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
     </row>
     <row r="244" spans="1:4">
@@ -5347,7 +5350,7 @@
         <v>261</v>
       </c>
       <c r="D244" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
     </row>
     <row r="245" spans="1:4">
@@ -5361,7 +5364,7 @@
         <v>261</v>
       </c>
       <c r="D245" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
     </row>
     <row r="246" spans="1:4">
@@ -5375,7 +5378,7 @@
         <v>261</v>
       </c>
       <c r="D246" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
     </row>
     <row r="247" spans="1:4">
@@ -5389,7 +5392,7 @@
         <v>261</v>
       </c>
       <c r="D247" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
     </row>
     <row r="248" spans="1:4">
@@ -5400,10 +5403,10 @@
         <v>261</v>
       </c>
       <c r="C248" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="D248" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
     </row>
     <row r="249" spans="1:4">
@@ -5417,7 +5420,7 @@
         <v>261</v>
       </c>
       <c r="D249" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
     </row>
     <row r="250" spans="1:4">
@@ -5428,10 +5431,10 @@
         <v>261</v>
       </c>
       <c r="C250" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D250" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
     </row>
     <row r="251" spans="1:4">
@@ -5442,10 +5445,10 @@
         <v>259</v>
       </c>
       <c r="C251" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D251" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
     </row>
     <row r="252" spans="1:4">
@@ -5459,7 +5462,7 @@
         <v>260</v>
       </c>
       <c r="D252" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
     </row>
     <row r="253" spans="1:4">
@@ -5473,7 +5476,7 @@
         <v>260</v>
       </c>
       <c r="D253" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
     </row>
     <row r="254" spans="1:4">
@@ -5487,7 +5490,7 @@
         <v>260</v>
       </c>
       <c r="D254" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
     </row>
     <row r="255" spans="1:4">
@@ -5501,7 +5504,7 @@
         <v>260</v>
       </c>
       <c r="D255" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
     </row>
     <row r="256" spans="1:4">
@@ -5515,7 +5518,7 @@
         <v>260</v>
       </c>
       <c r="D256" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
     </row>
   </sheetData>

</xml_diff>